<commit_message>
Updated readme and code fix
</commit_message>
<xml_diff>
--- a/docs/Evaluation_Test_Set.xlsx
+++ b/docs/Evaluation_Test_Set.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Haeron Projects\EY Case Study\acme-agent\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14806120-5EBB-4FCA-8090-398530490056}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B543337C-1986-4656-A4C6-C984CF2AF3BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,10 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="63">
-  <si>
-    <t>Test ID</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="60">
   <si>
     <t>User Role</t>
   </si>
@@ -41,9 +38,6 @@
     <t>RBAC Expected</t>
   </si>
   <si>
-    <t>Recommended Next Action?</t>
-  </si>
-  <si>
     <t>Expected Result</t>
   </si>
   <si>
@@ -53,9 +47,6 @@
     <t>Comments</t>
   </si>
   <si>
-    <t>TC-01</t>
-  </si>
-  <si>
     <t>support_user</t>
   </si>
   <si>
@@ -71,94 +62,49 @@
     <t>Allowed</t>
   </si>
   <si>
-    <t>N/A</t>
-  </si>
-  <si>
     <t>Returns Orion Financial open issues from PostgreSQL</t>
   </si>
   <si>
     <t>Pass</t>
   </si>
   <si>
-    <t>TC-02</t>
-  </si>
-  <si>
-    <t>customer_lookup + open_customer_issues + issue_history + recommended_next_actions + Executive Escalation Summary</t>
-  </si>
-  <si>
     <t>Grounded executive summary</t>
   </si>
   <si>
-    <t>TC-03</t>
-  </si>
-  <si>
     <t>sales_user</t>
   </si>
   <si>
     <t>Update Orion Financial issue status to Closed</t>
   </si>
   <si>
-    <t>update_issue_status (Local Tool)</t>
-  </si>
-  <si>
     <t>Denied</t>
   </si>
   <si>
     <t>Access denied by RBAC</t>
   </si>
   <si>
-    <t>TC-04</t>
-  </si>
-  <si>
     <t>admin</t>
   </si>
   <si>
     <t>Status updated</t>
   </si>
   <si>
-    <t>TC-05</t>
-  </si>
-  <si>
     <t>Who is the account manager for GreenWave Energy?</t>
   </si>
   <si>
     <t>customer_lookup (MCP)</t>
   </si>
   <si>
-    <t>Returns customer details</t>
-  </si>
-  <si>
-    <t>TC-06</t>
-  </si>
-  <si>
     <t>Show issue history for Nova Retail Ltd</t>
   </si>
   <si>
-    <t>issue_history (MCP)</t>
-  </si>
-  <si>
     <t>Returns issue history</t>
   </si>
   <si>
-    <t>TC-07</t>
-  </si>
-  <si>
     <t>What is the recommended next action for BluePeak Logistics?</t>
   </si>
   <si>
-    <t>recommended_next_actions (MCP)</t>
-  </si>
-  <si>
-    <t>Returns pending next action</t>
-  </si>
-  <si>
-    <t>TC-08</t>
-  </si>
-  <si>
     <t>Summarise the current situation for Vertex Manufacturing</t>
-  </si>
-  <si>
-    <t>customer_lookup + open_customer_issues + issue_history + Executive Escalation Summary</t>
   </si>
   <si>
     <t>Grounded summary</t>
@@ -195,33 +141,6 @@
 Issue 15 — Customer Onboarding Failure
 Priority: Medium
 Status: Open</t>
-  </si>
-  <si>
-    <t>Executive Escalation Summary: Orion Financial
-Executive Summary
-Orion Financial currently has three open issues affecting core financial workflows: loan approvals, fraud detection alerts, and customer onboarding. All three have been reproduced by Support and escalated to Engineering, with root causes identified and permanent fixes reportedly in progress. The most critical item is Loan Approval Workflow Stuck, which is blocking loan applications from moving out of pending status.
-Customer Health
-Customer health appears at risk based on the volume and severity of open issues. The portfolio includes one Critical, one High, and one Medium priority issue, all still open.
-Open Issues
-Issue 13 — Loan Approval Workflow Stuck
-Priority: Critical
-Status: Open
-Issue 14 — Fraud Detection Alerts Missing
-Priority: High
-Status: Open
-Issue 15 — Customer Onboarding Failure
-Priority: Medium
-Status: Open
-Existing Next Actions
-For each issue:
-Action: Schedule a customer review call and provide an implementation update.
-Owner: Support Team
-Status: Pending
-Business Risk
-Business risk is high because the issues affect lending, fraud monitoring, and onboarding workflows.
-Overall Priority
-Critical
-If you want, I can also give you the history or next action for any of these issues.</t>
   </si>
   <si>
     <t>Current situation for Vertex Manufacturing
@@ -272,7 +191,75 @@
     <t>The account manager for GreenWave Energy is James Walker.</t>
   </si>
   <si>
-    <t xml:space="preserve"> What is Executive escalation summary Orion Financial</t>
+    <t xml:space="preserve"> What is Executive escalation summary Nova retail</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Executive Escalation Summary</t>
+  </si>
+  <si>
+    <t>Customer issue issue is called and agent responded with issues for Orion Financial</t>
+  </si>
+  <si>
+    <t>Executive escalation summary for Nova Retail:
+Overall Priority: Critical
+Customer Health / Executive Summary: No information available.
+Open Issues
+Customer Portal Login Failure — Critical, Open
+Multiple users cannot log in to the customer portal.
+Engineering has identified the root cause and a permanent fix is being implemented.
+Payment Gateway Timeout — High, Open
+Customers are experiencing timeout errors during online checkout.
+Engineering has identified the root cause and a permanent fix is being implemented.
+Inventory Synchronization Failure — Medium, Open
+Warehouse stock levels are not synchronizing with the online store.
+Engineering has identified the root cause and a permanent fix is being implemented.
+Existing Next Actions
+Payment Gateway Timeout: schedule a customer review call and provide an implementation update.
+Inventory Synchronization Failure: schedule a customer review call and provide an implementation update.
+Customer Portal Login Failure: check shipment system logs.
+AI Recommended Next Steps
+Confirm ownership and timing for the pending customer review calls on the Payment Gateway Timeout and Inventory Synchronization Failure issues.
+Validate whether “check shipment system logs” is the correct next step for Customer Portal Login Failure.
+Consolidate the three incidents into a single executive-facing customer update.</t>
+  </si>
+  <si>
+    <t>Customer escallation summary tool was called and result was generated with next actions from the table and also AI generated next steps as expected</t>
+  </si>
+  <si>
+    <t>Issue update was done as the user was admin and return succes message</t>
+  </si>
+  <si>
+    <t>Customer lookup tool was called and account manager details were returned</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer issue, open issues and issue history tools were called and all the open issues were returned properly </t>
+  </si>
+  <si>
+    <t>Customer lookup, Open customer issue tool and recommended next action tools were called and next actions for all opened issues was returned</t>
+  </si>
+  <si>
+    <t>customer loolup, open customer issues and customer escalation summary was called and the summary for Vertex manufacturing was returned succefully</t>
+  </si>
+  <si>
+    <t>Returns Account manager details</t>
+  </si>
+  <si>
+    <t>Returns  next actions</t>
+  </si>
+  <si>
+    <t>Access was denied for the sales user to update issue table</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cusomter_issue, open_issues and issue_history </t>
+  </si>
+  <si>
+    <t>Customer lookup, Open customer issue tool</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer loolup, open customer issues and customer escalation summary </t>
+  </si>
+  <si>
+    <t>ID</t>
   </si>
 </sst>
 </file>
@@ -621,301 +608,294 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:J9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="52.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="52.109375" customWidth="1"/>
-    <col min="9" max="9" width="44.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="52.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="52.140625" customWidth="1"/>
+    <col min="5" max="5" width="29.5703125" customWidth="1"/>
+    <col min="7" max="7" width="17.5703125" customWidth="1"/>
+    <col min="8" max="8" width="44.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="106.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I3" t="s">
+        <v>14</v>
+      </c>
+      <c r="J3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H4" t="s">
+        <v>19</v>
+      </c>
+      <c r="I4" t="s">
+        <v>14</v>
+      </c>
+      <c r="J4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" t="s">
+        <v>12</v>
+      </c>
+      <c r="H6" t="s">
         <v>53</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="1" t="s">
+      <c r="I6" t="s">
+        <v>14</v>
+      </c>
+      <c r="J6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7">
         <v>6</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" t="s">
+        <v>12</v>
+      </c>
+      <c r="H7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I7" t="s">
+        <v>14</v>
+      </c>
+      <c r="J7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="210" x14ac:dyDescent="0.25">
+      <c r="A8">
         <v>7</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="B8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8" t="s">
+        <v>57</v>
+      </c>
+      <c r="F8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H8" t="s">
+        <v>54</v>
+      </c>
+      <c r="I8" t="s">
+        <v>14</v>
+      </c>
+      <c r="J8" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A9">
         <v>8</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" ht="201.6" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E9" t="s">
+        <v>58</v>
+      </c>
+      <c r="F9" t="s">
         <v>11</v>
       </c>
-      <c r="C2" t="s">
+      <c r="G9" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="H9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I9" t="s">
         <v>14</v>
       </c>
-      <c r="G2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I2" t="s">
-        <v>17</v>
-      </c>
-      <c r="J2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>62</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4" t="s">
-        <v>57</v>
-      </c>
-      <c r="E4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G4" t="s">
-        <v>26</v>
-      </c>
-      <c r="H4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I4" t="s">
-        <v>27</v>
-      </c>
-      <c r="J4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" t="s">
-        <v>59</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="E5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F5" t="s">
-        <v>14</v>
-      </c>
-      <c r="G5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H5" t="s">
-        <v>16</v>
-      </c>
-      <c r="I5" t="s">
-        <v>30</v>
-      </c>
-      <c r="J5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>31</v>
-      </c>
-      <c r="B6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" t="s">
-        <v>32</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="E6" t="s">
-        <v>33</v>
-      </c>
-      <c r="F6" t="s">
-        <v>14</v>
-      </c>
-      <c r="G6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H6" t="s">
-        <v>16</v>
-      </c>
-      <c r="I6" t="s">
-        <v>34</v>
-      </c>
-      <c r="J6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" t="s">
-        <v>36</v>
-      </c>
-      <c r="E7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F7" t="s">
-        <v>14</v>
-      </c>
-      <c r="G7" t="s">
-        <v>15</v>
-      </c>
-      <c r="H7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I7" t="s">
-        <v>38</v>
-      </c>
-      <c r="J7" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" t="s">
-        <v>40</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="E8" t="s">
-        <v>41</v>
-      </c>
-      <c r="F8" t="s">
-        <v>14</v>
-      </c>
-      <c r="G8" t="s">
-        <v>15</v>
-      </c>
-      <c r="H8" t="s">
-        <v>14</v>
-      </c>
-      <c r="I8" t="s">
-        <v>42</v>
-      </c>
-      <c r="J8" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>43</v>
-      </c>
-      <c r="B9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" t="s">
-        <v>44</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="E9" t="s">
-        <v>45</v>
-      </c>
-      <c r="F9" t="s">
-        <v>14</v>
-      </c>
-      <c r="G9" t="s">
-        <v>15</v>
-      </c>
-      <c r="H9" t="s">
-        <v>14</v>
-      </c>
-      <c r="I9" t="s">
-        <v>46</v>
-      </c>
       <c r="J9" t="s">
-        <v>18</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -926,36 +906,36 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>52</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>